<commit_message>
modified:   excel_data/Innovation_Fund_Projects_data - 120626.xlsx 	modified:   public/data/projects.json
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 120626.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 120626.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cmeurope-my.sharepoint.com/personal/salman_muhammad_cmeurope_org/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1965" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EB866FB-CDF0-4B08-886C-B125D881B4FA}"/>
+  <xr:revisionPtr revIDLastSave="1966" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE30B954-1CC2-40C2-BC7D-7914E21575A6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1174" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1174" uniqueCount="492">
   <si>
     <t>Status</t>
   </si>
@@ -1524,6 +1524,9 @@
   </si>
   <si>
     <t>The project applies oxyfuel combustion and a CO₂ compression and purification unit (CPU) at the Holcim Lägerdorf cement plant to capture approximately 1.3 Mt CO₂ per year. Captured CO₂ is then processed through a thyssenkrupp/Linde CPU and utilised as a feedstock for the production of industrial chemicals, including methanol and plastic precursors, enabling CCU-based carbon conversion.</t>
+  </si>
+  <si>
+    <t>Vow Green Metals</t>
   </si>
 </sst>
 </file>
@@ -7961,7 +7964,7 @@
         <v>9</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>192</v>
+        <v>491</v>
       </c>
       <c r="G61" s="6" t="s">
         <v>192</v>
@@ -8312,6 +8315,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100052CBA820BEBCD468114CF62615C95D9" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="41d93ad2b4fecab14cfdaed9255371f8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ba695df1-2cef-45b3-b38e-525c8136ab22" xmlns:ns3="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="59a815193907c452009623866744c535" ns2:_="" ns3:_="">
     <xsd:import namespace="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
@@ -8552,27 +8575,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82507086-9DCD-4197-A4F6-ECCED658E0D9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8589,29 +8617,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
modified:   excel_data/Innovation_Fund_Projects_data - 120626.xlsx 	modified:   public/data/meta.json 	modified:   public/data/projects.json
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 120626.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 120626.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cmeurope-my.sharepoint.com/personal/salman_muhammad_cmeurope_org/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1966" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE30B954-1CC2-40C2-BC7D-7914E21575A6}"/>
+  <xr:revisionPtr revIDLastSave="1973" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{164D9154-FC1A-46A4-A5AF-5583A80CF09C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -410,9 +410,6 @@
     <t>eM-Rhone</t>
   </si>
   <si>
-    <t>Elyse Energy</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://ec.europa.eu/assets/cinea/project_fiches/innovation_fund/101133147.pdf </t>
   </si>
   <si>
@@ -1076,12 +1073,6 @@
     <t>GIE OSIRIS</t>
   </si>
   <si>
-    <t>eM-Rhône is a French carbon capture and utilisation project led by Elyse Energy. It combines renewable hydrogen production on the Roches-Roussillon chemical platform in Salaise-sur-Sanne with carbon dioxide captured at Holcim/Lafarge’s cement plant in Le Teil, Ardèche, and transported by rail to the methanol site. The project is designed around 170 MW of PEM electrolysis, about 27 kt/year of hydrogen production, and about 195 kt/year of CO₂ use to produce large-scale e-methanol for chemical and maritime markets.</t>
-  </si>
-  <si>
-    <t>The project captures concentrated CO₂ from the Le Teil cement plant using a fully electric cryogenic capture scheme, liquefies and transports the CO₂ by rail to Salaise-sur-Sanne, then receives, stores, regasifies and purifies the CO₂ before reaction with hydrogen produced on site by 170 MW PEM electrolysis. The hydrogen is compressed and purified, then combined with the purified CO₂ in a methanol synthesis unit, followed by intermediate storage and final methanol storage via the adjacent TEPSA logistics system. The updated Innovation Fund factsheet gives 195 kt/year CO₂ input, 27 kt/year hydrogen production and 138 kt/year methanol output; Elyse’s project page still states 150 kt/year methanol.</t>
-  </si>
-  <si>
     <t>Usine Lafarge, 07220 Viviers, France</t>
   </si>
   <si>
@@ -1527,6 +1518,15 @@
   </si>
   <si>
     <t>Vow Green Metals</t>
+  </si>
+  <si>
+    <t>Elyse Energy, Lafarge (Holcim)</t>
+  </si>
+  <si>
+    <t>eM-Rhône is a joint venture of Elyse Energy and Lafarge Cement (Holcim). It combines renewable hydrogen production on the Roches-Roussillon chemical platform in Salaise-sur-Sanne with CO₂ captured at Holcim/Lafarge’s cement plant in Le Teil, Ardèche, and transported by rail to the methanol site. The project is designed around 170 MW of PEM electrolysis, about 27 kt/year of hydrogen production, and about 195 kt/year of CO₂ use to produce large-scale e-methanol for chemical and maritime markets.</t>
+  </si>
+  <si>
+    <t>The project captures concentrated CO₂ from the Le Teil cement plant using a fully electric cryogenic capture scheme, liquefies and transports the CO₂ by rail to Salaise-sur-Sanne, then receives, stores, regasifies and purifies the CO₂ before reaction with hydrogen produced on site by 170 MW PEM electrolysis. The hydrogen is compressed and purified, then combined with the purified CO₂ in a methanol synthesis unit, followed by intermediate storage and final methanol storage via the adjacent TEPSA logistics system. The updated Innovation Fund factsheet gives 195 kt/year CO₂ input, 27 kt/year hydrogen production and 138 kt/year methanol output.</t>
   </si>
 </sst>
 </file>
@@ -1883,7 +1883,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2097,6 +2097,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2493,10 +2496,10 @@
         <v>37</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>38</v>
@@ -2597,7 +2600,7 @@
         <v>220123498</v>
       </c>
       <c r="U2" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V2" s="46">
         <v>57.062100000000001</v>
@@ -2612,19 +2615,19 @@
         <v>95</v>
       </c>
       <c r="Z2" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA2" s="47" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AB2" s="41" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="AC2" s="41" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="AD2" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="3" spans="1:30" ht="114" x14ac:dyDescent="0.3">
@@ -2632,10 +2635,10 @@
         <v>96</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C3" s="40" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>70</v>
@@ -2644,10 +2647,10 @@
         <v>19</v>
       </c>
       <c r="F3" s="40" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G3" s="40" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H3" s="48">
         <v>0.12330000000000001</v>
@@ -2689,7 +2692,7 @@
         <v>31238542</v>
       </c>
       <c r="U3" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V3" s="46">
         <v>44.464755134852901</v>
@@ -2701,22 +2704,22 @@
         <v>57</v>
       </c>
       <c r="Y3" s="41" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="Z3" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA3" s="47" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AB3" s="41" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="AC3" s="41" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="AD3" s="38" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="4" spans="1:30" ht="125.4" x14ac:dyDescent="0.3">
@@ -2724,10 +2727,10 @@
         <v>59</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>103</v>
@@ -2736,10 +2739,10 @@
         <v>15</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H4" s="50" t="s">
         <v>54</v>
@@ -2781,7 +2784,7 @@
         <v>3168000</v>
       </c>
       <c r="U4" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V4" s="54">
         <v>43.327720234653299</v>
@@ -2793,19 +2796,19 @@
         <v>57</v>
       </c>
       <c r="Y4" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="Z4" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="AA4" s="47" t="s">
+        <v>235</v>
+      </c>
+      <c r="AB4" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="Z4" s="7" t="s">
-        <v>462</v>
-      </c>
-      <c r="AA4" s="47" t="s">
-        <v>236</v>
-      </c>
-      <c r="AB4" s="7" t="s">
+      <c r="AC4" s="7" t="s">
         <v>228</v>
-      </c>
-      <c r="AC4" s="7" t="s">
-        <v>229</v>
       </c>
       <c r="AD4" s="12" t="s">
         <v>2</v>
@@ -2816,13 +2819,13 @@
         <v>78</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C5" s="40" t="s">
         <v>69</v>
       </c>
       <c r="D5" s="41" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="E5" s="40" t="s">
         <v>5</v>
@@ -2858,7 +2861,7 @@
         <v>54</v>
       </c>
       <c r="P5" s="44" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="Q5" s="44">
         <v>2030</v>
@@ -2873,7 +2876,7 @@
         <v>145000000</v>
       </c>
       <c r="U5" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V5" s="46">
         <v>46.809800000000003</v>
@@ -2885,22 +2888,22 @@
         <v>57</v>
       </c>
       <c r="Y5" s="41" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="Z5" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA5" s="47" t="s">
+        <v>240</v>
+      </c>
+      <c r="AB5" s="41" t="s">
         <v>241</v>
       </c>
-      <c r="AB5" s="41" t="s">
+      <c r="AC5" s="41" t="s">
         <v>242</v>
       </c>
-      <c r="AC5" s="41" t="s">
-        <v>243</v>
-      </c>
       <c r="AD5" s="14" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="6" spans="1:30" ht="125.4" x14ac:dyDescent="0.3">
@@ -2908,10 +2911,10 @@
         <v>96</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C6" s="40" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D6" s="41" t="s">
         <v>103</v>
@@ -2920,10 +2923,10 @@
         <v>8</v>
       </c>
       <c r="F6" s="40" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G6" s="40" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H6" s="48">
         <v>2.5999999999999999E-2</v>
@@ -2965,7 +2968,7 @@
         <v>7958244</v>
       </c>
       <c r="U6" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V6" s="39" t="s">
         <v>54</v>
@@ -2974,25 +2977,25 @@
         <v>54</v>
       </c>
       <c r="X6" s="39" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y6" s="41" t="s">
         <v>54</v>
       </c>
       <c r="Z6" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA6" s="47" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="AB6" s="41" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="AC6" s="41" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="AD6" s="37" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="7" spans="1:30" ht="91.2" x14ac:dyDescent="0.3">
@@ -3057,7 +3060,7 @@
         <v>189694949</v>
       </c>
       <c r="U7" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V7" s="46">
         <v>43.232830995956597</v>
@@ -3069,22 +3072,22 @@
         <v>89</v>
       </c>
       <c r="Y7" s="41" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Z7" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA7" s="47" t="s">
+        <v>248</v>
+      </c>
+      <c r="AB7" s="41" t="s">
+        <v>247</v>
+      </c>
+      <c r="AC7" s="41" t="s">
         <v>249</v>
       </c>
-      <c r="AB7" s="41" t="s">
-        <v>248</v>
-      </c>
-      <c r="AC7" s="41" t="s">
-        <v>250</v>
-      </c>
       <c r="AD7" s="16" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="8" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -3134,7 +3137,7 @@
         <v>54</v>
       </c>
       <c r="P8" s="44" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="Q8" s="44">
         <v>2029</v>
@@ -3149,7 +3152,7 @@
         <v>115000000</v>
       </c>
       <c r="U8" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V8" s="46">
         <v>50.575420999999999</v>
@@ -3164,19 +3167,19 @@
         <v>82</v>
       </c>
       <c r="Z8" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA8" s="47" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="AB8" s="41" t="s">
         <v>83</v>
       </c>
       <c r="AC8" s="41" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="AD8" s="14" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="9" spans="1:30" ht="91.2" x14ac:dyDescent="0.3">
@@ -3184,22 +3187,22 @@
         <v>78</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="H9" s="50">
         <v>2.5819174</v>
@@ -3241,7 +3244,7 @@
         <v>169300000</v>
       </c>
       <c r="U9" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V9" s="54">
         <v>37.960247145532399</v>
@@ -3253,22 +3256,22 @@
         <v>57</v>
       </c>
       <c r="Y9" s="7" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="Z9" s="7" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="AA9" s="47" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="AB9" s="7" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="AC9" s="7" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="AD9" s="38" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="10" spans="1:30" ht="114" x14ac:dyDescent="0.3">
@@ -3276,22 +3279,22 @@
         <v>49</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D10" s="41" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="E10" s="40" t="s">
         <v>21</v>
       </c>
       <c r="F10" s="40" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G10" s="40" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H10" s="48" t="s">
         <v>54</v>
@@ -3345,19 +3348,19 @@
         <v>57</v>
       </c>
       <c r="Y10" s="41" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="Z10" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA10" s="47" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AB10" s="41" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="AC10" s="41" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="AD10" s="12" t="s">
         <v>2</v>
@@ -3368,10 +3371,10 @@
         <v>84</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C11" s="40" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D11" s="41" t="s">
         <v>103</v>
@@ -3380,10 +3383,10 @@
         <v>9</v>
       </c>
       <c r="F11" s="40" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G11" s="40" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H11" s="48" t="s">
         <v>54</v>
@@ -3425,7 +3428,7 @@
         <v>10206000</v>
       </c>
       <c r="U11" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V11" s="46">
         <v>59.592303479664103</v>
@@ -3434,25 +3437,25 @@
         <v>5.8029778441568904</v>
       </c>
       <c r="X11" s="39" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y11" s="41" t="s">
+        <v>299</v>
+      </c>
+      <c r="Z11" s="41" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA11" s="47" t="s">
+        <v>296</v>
+      </c>
+      <c r="AB11" s="41" t="s">
         <v>300</v>
       </c>
-      <c r="Z11" s="41" t="s">
-        <v>461</v>
-      </c>
-      <c r="AA11" s="47" t="s">
-        <v>297</v>
-      </c>
-      <c r="AB11" s="41" t="s">
+      <c r="AC11" s="41" t="s">
         <v>301</v>
       </c>
-      <c r="AC11" s="41" t="s">
-        <v>302</v>
-      </c>
       <c r="AD11" s="14" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="12" spans="1:30" ht="79.8" x14ac:dyDescent="0.3">
@@ -3460,7 +3463,7 @@
         <v>49</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>69</v>
@@ -3472,10 +3475,10 @@
         <v>11</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H12" s="50">
         <v>1.3</v>
@@ -3529,22 +3532,22 @@
         <v>57</v>
       </c>
       <c r="Y12" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="Z12" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA12" s="47" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="AB12" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="AC12" s="7" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="AD12" s="37" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="13" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -3621,22 +3624,22 @@
         <v>57</v>
       </c>
       <c r="Y13" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="Z13" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA13" s="57" t="s">
         <v>117</v>
       </c>
       <c r="AB13" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="AC13" s="7" t="s">
         <v>268</v>
       </c>
-      <c r="AC13" s="7" t="s">
-        <v>269</v>
-      </c>
       <c r="AD13" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="14" spans="1:30" ht="79.8" x14ac:dyDescent="0.3">
@@ -3644,10 +3647,10 @@
         <v>96</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>70</v>
@@ -3656,10 +3659,10 @@
         <v>19</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H14" s="50">
         <v>6.4000000000000001E-2</v>
@@ -3701,7 +3704,7 @@
         <v>23635998</v>
       </c>
       <c r="U14" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V14" s="54">
         <v>44.826999999999998</v>
@@ -3710,25 +3713,25 @@
         <v>11.614000000000001</v>
       </c>
       <c r="X14" s="49" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="Z14" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA14" s="47" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="AB14" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="AC14" s="7" t="s">
         <v>292</v>
       </c>
-      <c r="AC14" s="7" t="s">
-        <v>293</v>
-      </c>
       <c r="AD14" s="37" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="15" spans="1:30" ht="148.19999999999999" x14ac:dyDescent="0.3">
@@ -3736,7 +3739,7 @@
         <v>49</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>69</v>
@@ -3748,10 +3751,10 @@
         <v>5</v>
       </c>
       <c r="F15" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="G15" s="6" t="s">
         <v>122</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>123</v>
       </c>
       <c r="H15" s="50">
         <v>0.7</v>
@@ -3793,7 +3796,7 @@
         <v>119682059</v>
       </c>
       <c r="U15" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V15" s="54">
         <v>43.186100000000003</v>
@@ -3805,22 +3808,22 @@
         <v>57</v>
       </c>
       <c r="Y15" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="Z15" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA15" s="47" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="AB15" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="AC15" s="7" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="AD15" s="37" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="16" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -3828,7 +3831,7 @@
         <v>78</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>69</v>
@@ -3840,10 +3843,10 @@
         <v>22</v>
       </c>
       <c r="F16" s="40" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G16" s="40" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H16" s="48" t="s">
         <v>54</v>
@@ -3885,7 +3888,7 @@
         <v>146415990</v>
       </c>
       <c r="U16" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V16" s="46">
         <v>45.290985428950698</v>
@@ -3894,25 +3897,25 @@
         <v>25.1109549184484</v>
       </c>
       <c r="X16" s="39" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y16" s="41" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="Z16" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA16" s="47" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="AB16" s="41" t="s">
+        <v>306</v>
+      </c>
+      <c r="AC16" s="41" t="s">
         <v>307</v>
       </c>
-      <c r="AC16" s="41" t="s">
-        <v>308</v>
-      </c>
       <c r="AD16" s="15" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="17" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -3920,10 +3923,10 @@
         <v>59</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D17" s="41" t="s">
         <v>70</v>
@@ -3932,10 +3935,10 @@
         <v>6</v>
       </c>
       <c r="F17" s="40" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G17" s="40" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H17" s="58">
         <v>4.5999999999999999E-3</v>
@@ -3977,7 +3980,7 @@
         <v>30497000</v>
       </c>
       <c r="U17" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V17" s="39">
         <v>51.870851200822599</v>
@@ -3986,22 +3989,22 @@
         <v>4.30094696894741</v>
       </c>
       <c r="X17" s="39" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y17" s="41" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="Z17" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA17" s="59" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AB17" s="41" t="s">
+        <v>310</v>
+      </c>
+      <c r="AC17" s="41" t="s">
         <v>311</v>
-      </c>
-      <c r="AC17" s="41" t="s">
-        <v>312</v>
       </c>
       <c r="AD17" s="12" t="s">
         <v>2</v>
@@ -4012,7 +4015,7 @@
         <v>49</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C18" s="40" t="s">
         <v>69</v>
@@ -4024,10 +4027,10 @@
         <v>11</v>
       </c>
       <c r="F18" s="40" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G18" s="40" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H18" s="43">
         <v>1.3</v>
@@ -4069,7 +4072,7 @@
         <v>157000000</v>
       </c>
       <c r="U18" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V18" s="46">
         <v>52.489100000000001</v>
@@ -4081,22 +4084,22 @@
         <v>57</v>
       </c>
       <c r="Y18" s="41" t="s">
+        <v>144</v>
+      </c>
+      <c r="Z18" s="41" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA18" s="59" t="s">
         <v>145</v>
       </c>
-      <c r="Z18" s="41" t="s">
-        <v>461</v>
-      </c>
-      <c r="AA18" s="59" t="s">
-        <v>146</v>
-      </c>
       <c r="AB18" s="41" t="s">
+        <v>272</v>
+      </c>
+      <c r="AC18" s="41" t="s">
         <v>273</v>
       </c>
-      <c r="AC18" s="41" t="s">
-        <v>274</v>
-      </c>
       <c r="AD18" s="15" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="19" spans="1:30" ht="45.6" x14ac:dyDescent="0.3">
@@ -4161,7 +4164,7 @@
         <v>4265136</v>
       </c>
       <c r="U19" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V19" s="54">
         <v>50.569000000000003</v>
@@ -4176,10 +4179,10 @@
         <v>65</v>
       </c>
       <c r="Z19" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA19" s="47" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AB19" s="7" t="s">
         <v>66</v>
@@ -4196,22 +4199,22 @@
         <v>49</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D20" s="41" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>12</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="H20" s="50">
         <v>2.11</v>
@@ -4265,22 +4268,22 @@
         <v>57</v>
       </c>
       <c r="Y20" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="Z20" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="AA20" s="57" t="s">
         <v>167</v>
       </c>
-      <c r="Z20" s="7" t="s">
-        <v>463</v>
-      </c>
-      <c r="AA20" s="57" t="s">
-        <v>168</v>
-      </c>
       <c r="AB20" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="AC20" s="7" t="s">
         <v>315</v>
       </c>
-      <c r="AC20" s="7" t="s">
-        <v>316</v>
-      </c>
       <c r="AD20" s="17" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="21" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -4288,13 +4291,13 @@
         <v>84</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>15</v>
@@ -4303,7 +4306,7 @@
         <v>114</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H21" s="60">
         <v>0.63600000000000001</v>
@@ -4333,10 +4336,10 @@
         <v>2025</v>
       </c>
       <c r="Q21" s="52" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="R21" s="52" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="S21" s="49" t="s">
         <v>81</v>
@@ -4345,7 +4348,7 @@
         <v>25400000</v>
       </c>
       <c r="U21" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V21" s="54">
         <v>41.352637812781921</v>
@@ -4357,22 +4360,22 @@
         <v>89</v>
       </c>
       <c r="Y21" s="41" t="s">
+        <v>316</v>
+      </c>
+      <c r="Z21" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="AA21" s="47" t="s">
+        <v>318</v>
+      </c>
+      <c r="AB21" s="7" t="s">
         <v>317</v>
       </c>
-      <c r="Z21" s="7" t="s">
-        <v>463</v>
-      </c>
-      <c r="AA21" s="47" t="s">
-        <v>319</v>
-      </c>
-      <c r="AB21" s="7" t="s">
-        <v>318</v>
-      </c>
       <c r="AC21" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AD21" s="15" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="22" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -4380,10 +4383,10 @@
         <v>59</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="C22" s="40" t="s">
         <v>169</v>
-      </c>
-      <c r="C22" s="40" t="s">
-        <v>170</v>
       </c>
       <c r="D22" s="41" t="s">
         <v>103</v>
@@ -4392,10 +4395,10 @@
         <v>19</v>
       </c>
       <c r="F22" s="40" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G22" s="40" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H22" s="56">
         <v>1.7904E-2</v>
@@ -4446,25 +4449,25 @@
         <v>13.253440646806</v>
       </c>
       <c r="X22" s="39" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y22" s="62" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="Z22" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA22" s="47" t="s">
+        <v>319</v>
+      </c>
+      <c r="AB22" s="41" t="s">
         <v>320</v>
       </c>
-      <c r="AB22" s="41" t="s">
+      <c r="AC22" s="41" t="s">
         <v>321</v>
       </c>
-      <c r="AC22" s="41" t="s">
-        <v>322</v>
-      </c>
       <c r="AD22" s="37" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="23" spans="1:30" ht="136.80000000000001" x14ac:dyDescent="0.3">
@@ -4472,22 +4475,22 @@
         <v>96</v>
       </c>
       <c r="B23" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>162</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>163</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>20</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H23" s="50">
         <v>0.56499999999999995</v>
@@ -4541,22 +4544,22 @@
         <v>57</v>
       </c>
       <c r="Y23" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="Z23" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA23" s="47" t="s">
+        <v>324</v>
+      </c>
+      <c r="AB23" s="7" t="s">
         <v>325</v>
       </c>
-      <c r="AB23" s="7" t="s">
+      <c r="AC23" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="AC23" s="7" t="s">
-        <v>327</v>
-      </c>
       <c r="AD23" s="15" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="24" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -4564,10 +4567,10 @@
         <v>78</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>103</v>
@@ -4576,10 +4579,10 @@
         <v>5</v>
       </c>
       <c r="F24" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="G24" s="7" t="s">
         <v>334</v>
-      </c>
-      <c r="G24" s="7" t="s">
-        <v>335</v>
       </c>
       <c r="H24" s="50">
         <v>0.2</v>
@@ -4630,25 +4633,25 @@
         <v>1.1835034670687401</v>
       </c>
       <c r="X24" s="49" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y24" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z24" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA24" s="47" t="s">
         <v>338</v>
       </c>
-      <c r="Z24" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="AA24" s="47" t="s">
-        <v>339</v>
-      </c>
       <c r="AB24" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="AC24" s="7" t="s">
         <v>336</v>
       </c>
-      <c r="AC24" s="7" t="s">
-        <v>337</v>
-      </c>
       <c r="AD24" s="38" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="25" spans="1:30" ht="91.2" x14ac:dyDescent="0.3">
@@ -4656,7 +4659,7 @@
         <v>78</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>69</v>
@@ -4668,10 +4671,10 @@
         <v>19</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="H25" s="50">
         <v>1</v>
@@ -4713,7 +4716,7 @@
         <v>216000000</v>
       </c>
       <c r="U25" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V25" s="54">
         <v>45.515127894849797</v>
@@ -4722,25 +4725,25 @@
         <v>10.343124922954001</v>
       </c>
       <c r="X25" s="49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y25" s="7" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="Z25" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA25" s="47" t="s">
+        <v>329</v>
+      </c>
+      <c r="AB25" s="7" t="s">
         <v>330</v>
       </c>
-      <c r="AB25" s="7" t="s">
+      <c r="AC25" s="7" t="s">
         <v>331</v>
       </c>
-      <c r="AC25" s="7" t="s">
-        <v>332</v>
-      </c>
       <c r="AD25" s="15" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="26" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -4748,10 +4751,10 @@
         <v>49</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>103</v>
@@ -4760,7 +4763,7 @@
         <v>9</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G26" s="6" t="s">
         <v>55</v>
@@ -4805,7 +4808,7 @@
         <v>40000000</v>
       </c>
       <c r="U26" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V26" s="49">
         <v>59.121267699503399</v>
@@ -4814,28 +4817,28 @@
         <v>9.6300609243118291</v>
       </c>
       <c r="X26" s="49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y26" s="7" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="Z26" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="AA26" s="57" t="s">
+        <v>185</v>
+      </c>
+      <c r="AB26" s="7" t="s">
+        <v>463</v>
+      </c>
+      <c r="AC26" s="7" t="s">
         <v>464</v>
       </c>
-      <c r="AA26" s="57" t="s">
-        <v>186</v>
-      </c>
-      <c r="AB26" s="7" t="s">
-        <v>466</v>
-      </c>
-      <c r="AC26" s="7" t="s">
-        <v>467</v>
-      </c>
       <c r="AD26" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
-    <row r="27" spans="1:30" ht="125.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A27" s="39" t="s">
         <v>49</v>
       </c>
@@ -4851,11 +4854,11 @@
       <c r="E27" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="F27" s="40" t="s">
-        <v>119</v>
+      <c r="F27" s="2" t="s">
+        <v>489</v>
       </c>
       <c r="G27" s="40" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="H27" s="48">
         <v>0.23252429999999999</v>
@@ -4909,22 +4912,22 @@
         <v>57</v>
       </c>
       <c r="Y27" s="41" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="Z27" s="41" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="AA27" s="59" t="s">
-        <v>120</v>
-      </c>
-      <c r="AB27" s="41" t="s">
-        <v>341</v>
+        <v>119</v>
+      </c>
+      <c r="AB27" s="72" t="s">
+        <v>490</v>
       </c>
       <c r="AC27" s="41" t="s">
-        <v>342</v>
+        <v>491</v>
       </c>
       <c r="AD27" s="38" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="28" spans="1:30" ht="91.2" x14ac:dyDescent="0.3">
@@ -4935,10 +4938,10 @@
         <v>100</v>
       </c>
       <c r="C28" s="40" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D28" s="41" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="E28" s="40" t="s">
         <v>17</v>
@@ -4989,7 +4992,7 @@
         <v>54000000</v>
       </c>
       <c r="U28" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V28" s="46">
         <v>54.992185868676003</v>
@@ -5001,22 +5004,22 @@
         <v>89</v>
       </c>
       <c r="Y28" s="41" t="s">
+        <v>341</v>
+      </c>
+      <c r="Z28" s="41" t="s">
+        <v>461</v>
+      </c>
+      <c r="AA28" s="47" t="s">
+        <v>342</v>
+      </c>
+      <c r="AB28" s="41" t="s">
+        <v>343</v>
+      </c>
+      <c r="AC28" s="41" t="s">
         <v>344</v>
       </c>
-      <c r="Z28" s="41" t="s">
-        <v>464</v>
-      </c>
-      <c r="AA28" s="47" t="s">
-        <v>345</v>
-      </c>
-      <c r="AB28" s="41" t="s">
-        <v>346</v>
-      </c>
-      <c r="AC28" s="41" t="s">
-        <v>347</v>
-      </c>
       <c r="AD28" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="29" spans="1:30" ht="114" x14ac:dyDescent="0.3">
@@ -5024,7 +5027,7 @@
         <v>49</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C29" s="40" t="s">
         <v>61</v>
@@ -5036,10 +5039,10 @@
         <v>11</v>
       </c>
       <c r="F29" s="40" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G29" s="40" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H29" s="43">
         <v>1.5</v>
@@ -5081,7 +5084,7 @@
         <v>228721666</v>
       </c>
       <c r="U29" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V29" s="46">
         <v>51.297800000000002</v>
@@ -5090,25 +5093,25 @@
         <v>7.0148000000000001</v>
       </c>
       <c r="X29" s="39" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y29" s="41" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="Z29" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA29" s="59" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AB29" s="41" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="AC29" s="41" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="AD29" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="30" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -5116,22 +5119,22 @@
         <v>113</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H30" s="60">
         <v>4.5999999999999999E-2</v>
@@ -5173,7 +5176,7 @@
         <v>29500000</v>
       </c>
       <c r="U30" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V30" s="49">
         <v>60.618241659279597</v>
@@ -5182,25 +5185,25 @@
         <v>16.891107915855802</v>
       </c>
       <c r="X30" s="49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y30" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="Z30" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA30" s="63" t="s">
+        <v>373</v>
+      </c>
+      <c r="AB30" s="7" t="s">
         <v>374</v>
       </c>
-      <c r="Z30" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="AA30" s="63" t="s">
-        <v>376</v>
-      </c>
-      <c r="AB30" s="7" t="s">
-        <v>377</v>
-      </c>
       <c r="AC30" s="7" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="AD30" s="38" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="31" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -5208,7 +5211,7 @@
         <v>49</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>69</v>
@@ -5265,7 +5268,7 @@
         <v>191000000</v>
       </c>
       <c r="U31" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V31" s="54">
         <v>51.618000000000002</v>
@@ -5277,22 +5280,22 @@
         <v>57</v>
       </c>
       <c r="Y31" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="Z31" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA31" s="64" t="s">
         <v>141</v>
       </c>
-      <c r="Z31" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="AA31" s="64" t="s">
-        <v>142</v>
-      </c>
       <c r="AB31" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="AC31" s="7" t="s">
         <v>290</v>
       </c>
-      <c r="AC31" s="7" t="s">
-        <v>291</v>
-      </c>
       <c r="AD31" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="32" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -5300,7 +5303,7 @@
         <v>49</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>69</v>
@@ -5312,10 +5315,10 @@
         <v>8</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="H32" s="50">
         <v>1</v>
@@ -5369,22 +5372,22 @@
         <v>57</v>
       </c>
       <c r="Y32" s="7" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="Z32" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA32" s="47" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="AB32" s="7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="AC32" s="7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AD32" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="33" spans="1:30" ht="91.2" x14ac:dyDescent="0.3">
@@ -5464,19 +5467,19 @@
         <v>73</v>
       </c>
       <c r="Z33" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA33" s="47" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="AB33" s="41" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="AC33" s="41" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="AD33" s="17" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="34" spans="1:30" ht="91.2" x14ac:dyDescent="0.3">
@@ -5484,19 +5487,19 @@
         <v>49</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C34" s="40" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D34" s="41" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="E34" s="40" t="s">
         <v>15</v>
       </c>
       <c r="F34" s="40" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G34" s="40"/>
       <c r="H34" s="48">
@@ -5539,7 +5542,7 @@
         <v>122900000</v>
       </c>
       <c r="U34" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V34" s="39">
         <v>43.151000000000003</v>
@@ -5548,25 +5551,25 @@
         <v>-7.6859999999999999</v>
       </c>
       <c r="X34" s="39" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y34" s="41" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="Z34" s="41" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="AA34" s="47" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AB34" s="41" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="AC34" s="41" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="AD34" s="37" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="35" spans="1:30" ht="114" x14ac:dyDescent="0.3">
@@ -5577,10 +5580,10 @@
         <v>97</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>17</v>
@@ -5589,7 +5592,7 @@
         <v>98</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="H35" s="50">
         <v>0.28144999999999998</v>
@@ -5646,16 +5649,16 @@
         <v>99</v>
       </c>
       <c r="Z35" s="7" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="AA35" s="47" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="AB35" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="AC35" s="7" t="s">
         <v>259</v>
-      </c>
-      <c r="AC35" s="7" t="s">
-        <v>260</v>
       </c>
       <c r="AD35" s="12" t="s">
         <v>2</v>
@@ -5669,7 +5672,7 @@
         <v>74</v>
       </c>
       <c r="C36" s="40" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="D36" s="7" t="s">
         <v>70</v>
@@ -5723,7 +5726,7 @@
         <v>159000000</v>
       </c>
       <c r="U36" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V36" s="54">
         <v>51.1339349</v>
@@ -5735,22 +5738,22 @@
         <v>57</v>
       </c>
       <c r="Y36" s="7" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="Z36" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA36" s="47" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="AB36" s="7" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="AC36" s="7" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="AD36" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="37" spans="1:30" ht="91.2" x14ac:dyDescent="0.3">
@@ -5758,22 +5761,22 @@
         <v>113</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>8</v>
       </c>
       <c r="F37" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="G37" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="H37" s="60">
         <v>5.0046999999999999E-3</v>
@@ -5815,7 +5818,7 @@
         <v>26498650</v>
       </c>
       <c r="U37" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V37" s="54">
         <v>50.529000000000003</v>
@@ -5827,22 +5830,22 @@
         <v>57</v>
       </c>
       <c r="Y37" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Z37" s="7" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="AA37" s="47" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="AB37" s="7" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="AC37" s="7" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="AD37" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="38" spans="1:30" ht="91.2" x14ac:dyDescent="0.3">
@@ -5850,7 +5853,7 @@
         <v>49</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C38" s="40" t="s">
         <v>69</v>
@@ -5862,10 +5865,10 @@
         <v>13</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H38" s="50">
         <v>0.68</v>
@@ -5907,7 +5910,7 @@
         <v>234000000</v>
       </c>
       <c r="U38" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V38" s="54">
         <v>38.129899999999999</v>
@@ -5919,22 +5922,22 @@
         <v>57</v>
       </c>
       <c r="Y38" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="Z38" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA38" s="47" t="s">
         <v>288</v>
       </c>
-      <c r="Z38" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="AA38" s="47" t="s">
-        <v>289</v>
-      </c>
       <c r="AB38" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="AC38" s="7" t="s">
         <v>286</v>
       </c>
-      <c r="AC38" s="7" t="s">
-        <v>287</v>
-      </c>
       <c r="AD38" s="38" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="39" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -5942,10 +5945,10 @@
         <v>96</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C39" s="40" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="D39" s="7" t="s">
         <v>70</v>
@@ -5954,7 +5957,7 @@
         <v>21</v>
       </c>
       <c r="F39" s="40" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G39" s="40"/>
       <c r="H39" s="48">
@@ -6006,22 +6009,22 @@
         <v>12.7671053619066</v>
       </c>
       <c r="X39" s="39" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y39" s="41" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Z39" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA39" s="47" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="AB39" s="41" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="AC39" s="41" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="AD39" s="13" t="s">
         <v>2</v>
@@ -6032,22 +6035,22 @@
         <v>49</v>
       </c>
       <c r="B40" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="C40" s="40" t="s">
         <v>153</v>
       </c>
-      <c r="C40" s="40" t="s">
-        <v>154</v>
-      </c>
       <c r="D40" s="41" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="E40" s="40" t="s">
         <v>13</v>
       </c>
       <c r="F40" s="40" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G40" s="40" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H40" s="48">
         <v>0.85799999999999998</v>
@@ -6089,7 +6092,7 @@
         <v>127000000</v>
       </c>
       <c r="U40" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V40" s="46">
         <v>37.916800000000002</v>
@@ -6101,22 +6104,22 @@
         <v>57</v>
       </c>
       <c r="Y40" s="41" t="s">
+        <v>155</v>
+      </c>
+      <c r="Z40" s="41" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA40" s="47" t="s">
         <v>156</v>
       </c>
-      <c r="Z40" s="41" t="s">
-        <v>461</v>
-      </c>
-      <c r="AA40" s="47" t="s">
-        <v>157</v>
-      </c>
       <c r="AB40" s="41" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="AC40" s="41" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="AD40" s="37" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="41" spans="1:30" ht="79.8" x14ac:dyDescent="0.3">
@@ -6181,7 +6184,7 @@
         <v>356900000</v>
       </c>
       <c r="U41" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V41" s="46">
         <v>51.368588000000003</v>
@@ -6196,19 +6199,19 @@
         <v>58</v>
       </c>
       <c r="Z41" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA41" s="47" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="AB41" s="41" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="AC41" s="41" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="AD41" s="17" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="42" spans="1:30" ht="79.8" x14ac:dyDescent="0.3">
@@ -6273,7 +6276,7 @@
         <v>117000000</v>
       </c>
       <c r="U42" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V42" s="54">
         <v>44.968299999999999</v>
@@ -6288,19 +6291,19 @@
         <v>92</v>
       </c>
       <c r="Z42" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA42" s="47" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="AB42" s="7" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="AC42" s="7" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="AD42" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="43" spans="1:30" ht="114" x14ac:dyDescent="0.3">
@@ -6308,19 +6311,19 @@
         <v>49</v>
       </c>
       <c r="B43" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="C43" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="C43" s="6" t="s">
-        <v>263</v>
-      </c>
       <c r="D43" s="41" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G43" s="6" t="s">
         <v>54</v>
@@ -6365,7 +6368,7 @@
         <v>118000000</v>
       </c>
       <c r="U43" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V43" s="54">
         <v>51.976999999999997</v>
@@ -6377,22 +6380,22 @@
         <v>57</v>
       </c>
       <c r="Y43" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Z43" s="7" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="AA43" s="63" t="s">
+        <v>263</v>
+      </c>
+      <c r="AB43" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="AB43" s="7" t="s">
+      <c r="AC43" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="AC43" s="7" t="s">
-        <v>266</v>
-      </c>
       <c r="AD43" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="44" spans="1:30" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -6457,7 +6460,7 @@
         <v>36000000</v>
       </c>
       <c r="U44" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V44" s="54">
         <v>50.406342306737002</v>
@@ -6469,22 +6472,22 @@
         <v>57</v>
       </c>
       <c r="Y44" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="Z44" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA44" s="47" t="s">
+        <v>377</v>
+      </c>
+      <c r="AB44" s="7" t="s">
+        <v>378</v>
+      </c>
+      <c r="AC44" s="7" t="s">
         <v>379</v>
       </c>
-      <c r="Z44" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="AA44" s="47" t="s">
-        <v>380</v>
-      </c>
-      <c r="AB44" s="7" t="s">
-        <v>381</v>
-      </c>
-      <c r="AC44" s="7" t="s">
-        <v>382</v>
-      </c>
       <c r="AD44" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="45" spans="1:30" ht="79.8" x14ac:dyDescent="0.3">
@@ -6492,19 +6495,19 @@
         <v>113</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>9</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="G45" s="6" t="s">
         <v>54</v>
@@ -6549,7 +6552,7 @@
         <v>13000000</v>
       </c>
       <c r="U45" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V45" s="49">
         <v>59.2181</v>
@@ -6558,25 +6561,25 @@
         <v>10.9298</v>
       </c>
       <c r="X45" s="49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y45" s="7" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="Z45" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AA45" s="47" t="s">
+        <v>380</v>
+      </c>
+      <c r="AB45" s="7" t="s">
         <v>383</v>
       </c>
-      <c r="AB45" s="7" t="s">
-        <v>386</v>
-      </c>
       <c r="AC45" s="7" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="AD45" s="37" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="46" spans="1:30" ht="114" x14ac:dyDescent="0.3">
@@ -6584,7 +6587,7 @@
         <v>49</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C46" s="40" t="s">
         <v>69</v>
@@ -6596,10 +6599,10 @@
         <v>13</v>
       </c>
       <c r="F46" s="40" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G46" s="40" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H46" s="48" t="s">
         <v>54</v>
@@ -6653,22 +6656,22 @@
         <v>57</v>
       </c>
       <c r="Y46" s="41" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="Z46" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA46" s="47" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="AB46" s="41" t="s">
+        <v>282</v>
+      </c>
+      <c r="AC46" s="41" t="s">
         <v>283</v>
       </c>
-      <c r="AC46" s="41" t="s">
-        <v>284</v>
-      </c>
       <c r="AD46" s="37" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="47" spans="1:30" ht="114" x14ac:dyDescent="0.3">
@@ -6679,7 +6682,7 @@
         <v>105</v>
       </c>
       <c r="C47" s="40" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D47" s="41" t="s">
         <v>103</v>
@@ -6688,10 +6691,10 @@
         <v>18</v>
       </c>
       <c r="F47" s="40" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="G47" s="40" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="H47" s="56">
         <v>1.55E-2</v>
@@ -6733,7 +6736,7 @@
         <v>8600000</v>
       </c>
       <c r="U47" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V47" s="46">
         <v>58.418889999999998</v>
@@ -6748,19 +6751,19 @@
         <v>106</v>
       </c>
       <c r="Z47" s="41" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="AA47" s="47" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="AB47" s="41" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="AC47" s="41" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="AD47" s="15" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="48" spans="1:30" ht="91.2" x14ac:dyDescent="0.3">
@@ -6768,7 +6771,7 @@
         <v>49</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C48" s="40" t="s">
         <v>51</v>
@@ -6780,10 +6783,10 @@
         <v>21</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="H48" s="50">
         <v>0.40600000000000003</v>
@@ -6825,7 +6828,7 @@
         <v>97000000</v>
       </c>
       <c r="U48" s="53" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="V48" s="49">
         <v>58.099057767351503</v>
@@ -6834,25 +6837,25 @@
         <v>11.861499508001399</v>
       </c>
       <c r="X48" s="49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y48" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="Z48" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA48" s="63" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AB48" s="7" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="AC48" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AD48" s="38" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="49" spans="1:30" ht="79.8" x14ac:dyDescent="0.3">
@@ -6863,7 +6866,7 @@
         <v>102</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D49" s="7" t="s">
         <v>103</v>
@@ -6872,10 +6875,10 @@
         <v>17</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="H49" s="60">
         <v>6.7077999999999999E-2</v>
@@ -6917,7 +6920,7 @@
         <v>40000000</v>
       </c>
       <c r="U49" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V49" s="54">
         <v>56.787056035485499</v>
@@ -6932,19 +6935,19 @@
         <v>104</v>
       </c>
       <c r="Z49" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA49" s="47" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="AB49" s="7" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="AC49" s="7" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="AD49" s="37" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="50" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -6952,22 +6955,22 @@
         <v>84</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H50" s="50">
         <v>0.24099999999999999</v>
@@ -6997,7 +7000,7 @@
         <v>19458418</v>
       </c>
       <c r="U50" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V50" s="54">
         <v>48.096166502584701</v>
@@ -7009,22 +7012,22 @@
         <v>89</v>
       </c>
       <c r="Y50" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="Z50" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="AA50" s="47" t="s">
+        <v>397</v>
+      </c>
+      <c r="AB50" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="AC50" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="Z50" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="AA50" s="47" t="s">
-        <v>400</v>
-      </c>
-      <c r="AB50" s="7" t="s">
-        <v>401</v>
-      </c>
-      <c r="AC50" s="7" t="s">
-        <v>402</v>
-      </c>
       <c r="AD50" s="15" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="51" spans="1:30" ht="91.2" x14ac:dyDescent="0.3">
@@ -7032,10 +7035,10 @@
         <v>78</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C51" s="40" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D51" s="41" t="s">
         <v>103</v>
@@ -7044,10 +7047,10 @@
         <v>5</v>
       </c>
       <c r="F51" s="40" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="G51" s="41" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="H51" s="48">
         <v>0.27411429999999998</v>
@@ -7101,22 +7104,22 @@
         <v>89</v>
       </c>
       <c r="Y51" s="41" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="Z51" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA51" s="47" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="AB51" s="41" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="AC51" s="41" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="AD51" s="15" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="52" spans="1:30" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -7127,7 +7130,7 @@
         <v>107</v>
       </c>
       <c r="C52" s="40" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D52" s="40" t="s">
         <v>70</v>
@@ -7181,7 +7184,7 @@
         <v>88286266</v>
       </c>
       <c r="U52" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V52" s="54">
         <v>60.306100000000001</v>
@@ -7196,7 +7199,7 @@
         <v>109</v>
       </c>
       <c r="Z52" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA52" s="47" t="s">
         <v>110</v>
@@ -7208,7 +7211,7 @@
         <v>112</v>
       </c>
       <c r="AD52" s="17" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="53" spans="1:30" ht="114" x14ac:dyDescent="0.3">
@@ -7216,10 +7219,10 @@
         <v>59</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="D53" s="41" t="s">
         <v>70</v>
@@ -7228,10 +7231,10 @@
         <v>12</v>
       </c>
       <c r="F53" s="40" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G53" s="40" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="H53" s="48">
         <v>1.72E-2</v>
@@ -7273,7 +7276,7 @@
         <v>3867988</v>
       </c>
       <c r="U53" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V53" s="46">
         <v>64.037112316635401</v>
@@ -7285,19 +7288,19 @@
         <v>57</v>
       </c>
       <c r="Y53" s="41" t="s">
+        <v>407</v>
+      </c>
+      <c r="Z53" s="41" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA53" s="47" t="s">
+        <v>408</v>
+      </c>
+      <c r="AB53" s="41" t="s">
         <v>410</v>
       </c>
-      <c r="Z53" s="41" t="s">
-        <v>461</v>
-      </c>
-      <c r="AA53" s="47" t="s">
+      <c r="AC53" s="41" t="s">
         <v>411</v>
-      </c>
-      <c r="AB53" s="41" t="s">
-        <v>413</v>
-      </c>
-      <c r="AC53" s="41" t="s">
-        <v>414</v>
       </c>
       <c r="AD53" s="11" t="s">
         <v>3</v>
@@ -7308,22 +7311,22 @@
         <v>113</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C54" s="40" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="D54" s="41" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="E54" s="40" t="s">
         <v>9</v>
       </c>
       <c r="F54" s="40" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="G54" s="41" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="H54" s="48">
         <v>0.16981750000000001</v>
@@ -7365,7 +7368,7 @@
         <v>40000000</v>
       </c>
       <c r="U54" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V54" s="46">
         <v>59.127044152710397</v>
@@ -7377,22 +7380,22 @@
         <v>89</v>
       </c>
       <c r="Y54" s="41" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="Z54" s="41" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA54" s="47" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="AB54" s="41" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="AC54" s="41" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="AD54" s="15" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="55" spans="1:30" ht="125.4" x14ac:dyDescent="0.3">
@@ -7400,22 +7403,22 @@
         <v>49</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C55" s="40" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D55" s="41" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="E55" s="40" t="s">
         <v>9</v>
       </c>
       <c r="F55" s="40" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G55" s="40" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="H55" s="48">
         <v>4.2</v>
@@ -7457,7 +7460,7 @@
         <v>225000000</v>
       </c>
       <c r="U55" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V55" s="39">
         <v>57.788622470324199</v>
@@ -7469,22 +7472,22 @@
         <v>89</v>
       </c>
       <c r="Y55" s="41" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="Z55" s="41" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="AA55" s="47" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AB55" s="41" t="s">
+        <v>270</v>
+      </c>
+      <c r="AC55" s="41" t="s">
         <v>271</v>
       </c>
-      <c r="AC55" s="41" t="s">
-        <v>272</v>
-      </c>
       <c r="AD55" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="56" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -7492,7 +7495,7 @@
         <v>113</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C56" s="40" t="s">
         <v>69</v>
@@ -7504,10 +7507,10 @@
         <v>5</v>
       </c>
       <c r="F56" s="40" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="G56" s="40" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="H56" s="48">
         <v>0.17</v>
@@ -7561,22 +7564,22 @@
         <v>57</v>
       </c>
       <c r="Y56" s="41" t="s">
+        <v>422</v>
+      </c>
+      <c r="Z56" s="41" t="s">
+        <v>459</v>
+      </c>
+      <c r="AA56" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="AB56" s="41" t="s">
+        <v>424</v>
+      </c>
+      <c r="AC56" s="41" t="s">
         <v>425</v>
       </c>
-      <c r="Z56" s="41" t="s">
-        <v>462</v>
-      </c>
-      <c r="AA56" s="47" t="s">
-        <v>426</v>
-      </c>
-      <c r="AB56" s="41" t="s">
-        <v>427</v>
-      </c>
-      <c r="AC56" s="41" t="s">
-        <v>428</v>
-      </c>
       <c r="AD56" s="37" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="57" spans="1:30" ht="79.8" x14ac:dyDescent="0.3">
@@ -7584,22 +7587,22 @@
         <v>49</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C57" s="40" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D57" s="41" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="E57" s="40" t="s">
         <v>15</v>
       </c>
       <c r="F57" s="40" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="G57" s="40" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="H57" s="48">
         <v>2</v>
@@ -7641,7 +7644,7 @@
         <v>205061582</v>
       </c>
       <c r="U57" s="45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V57" s="46">
         <v>40.8482802817337</v>
@@ -7653,22 +7656,22 @@
         <v>89</v>
       </c>
       <c r="Y57" s="41" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="Z57" s="41" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="AA57" s="59" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="AB57" s="41" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="AC57" s="41" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="AD57" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="58" spans="1:30" ht="102.6" x14ac:dyDescent="0.3">
@@ -7676,22 +7679,22 @@
         <v>84</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D58" s="7" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="E58" s="40" t="s">
         <v>13</v>
       </c>
       <c r="F58" s="40" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G58" s="40" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H58" s="56">
         <v>7.8E-2</v>
@@ -7745,22 +7748,22 @@
         <v>89</v>
       </c>
       <c r="Y58" s="41" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="Z58" s="41" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AA58" s="47" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="AB58" s="41" t="s">
+        <v>438</v>
+      </c>
+      <c r="AC58" s="41" t="s">
+        <v>439</v>
+      </c>
+      <c r="AD58" s="18" t="s">
         <v>441</v>
-      </c>
-      <c r="AC58" s="41" t="s">
-        <v>442</v>
-      </c>
-      <c r="AD58" s="18" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="59" spans="1:30" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -7768,10 +7771,10 @@
         <v>49</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D59" s="7" t="s">
         <v>103</v>
@@ -7780,10 +7783,10 @@
         <v>15</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H59" s="60">
         <v>8.5999999999999993E-2</v>
@@ -7834,25 +7837,25 @@
         <v>-8.2351799999999997</v>
       </c>
       <c r="X59" s="49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y59" s="7" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="Z59" s="7" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="AA59" s="57" t="s">
+        <v>211</v>
+      </c>
+      <c r="AB59" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="AC59" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="AB59" s="7" t="s">
-        <v>434</v>
-      </c>
-      <c r="AC59" s="7" t="s">
-        <v>213</v>
-      </c>
       <c r="AD59" s="38" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="60" spans="1:30" ht="79.8" x14ac:dyDescent="0.3">
@@ -7860,7 +7863,7 @@
         <v>78</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>69</v>
@@ -7872,10 +7875,10 @@
         <v>5</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H60" s="50">
         <v>1.2</v>
@@ -7929,22 +7932,22 @@
         <v>57</v>
       </c>
       <c r="Y60" s="7" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="Z60" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="AA60" s="47" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="AB60" s="7" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="AC60" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AD60" s="18" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="61" spans="1:30" ht="91.2" x14ac:dyDescent="0.3">
@@ -7952,22 +7955,22 @@
         <v>84</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C61" s="40" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>9</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H61" s="50">
         <v>0.1</v>
@@ -8009,7 +8012,7 @@
         <v>26200000</v>
       </c>
       <c r="U61" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V61" s="54">
         <v>59.242157075260003</v>
@@ -8018,25 +8021,25 @@
         <v>11.046906259539099</v>
       </c>
       <c r="X61" s="49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y61" s="7" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="Z61" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AA61" s="47" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="AB61" s="7" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="AC61" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AD61" s="15" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
   </sheetData>
@@ -8125,7 +8128,7 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="71" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B1" s="71"/>
     </row>
@@ -8151,10 +8154,10 @@
     </row>
     <row r="3" spans="1:14" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="30" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="C3" s="22"/>
       <c r="D3" s="20"/>
@@ -8171,10 +8174,10 @@
     </row>
     <row r="4" spans="1:14" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="35" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="C4" s="22"/>
       <c r="D4" s="20"/>
@@ -8191,10 +8194,10 @@
     </row>
     <row r="5" spans="1:14" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="34" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C5" s="22"/>
       <c r="D5" s="20"/>
@@ -8211,10 +8214,10 @@
     </row>
     <row r="6" spans="1:14" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="36" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C6" s="22"/>
       <c r="D6" s="20"/>
@@ -8234,7 +8237,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="C7" s="22"/>
       <c r="D7" s="20"/>
@@ -8254,7 +8257,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="C8" s="22"/>
       <c r="D8" s="20"/>
@@ -8271,10 +8274,10 @@
     </row>
     <row r="9" spans="1:14" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="33" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="C9" s="24"/>
       <c r="D9" s="25"/>
@@ -8315,17 +8318,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -8334,7 +8326,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100052CBA820BEBCD468114CF62615C95D9" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="41d93ad2b4fecab14cfdaed9255371f8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ba695df1-2cef-45b3-b38e-525c8136ab22" xmlns:ns3="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="59a815193907c452009623866744c535" ns2:_="" ns3:_="">
     <xsd:import namespace="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
@@ -8575,24 +8567,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -8600,7 +8586,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82507086-9DCD-4197-A4F6-ECCED658E0D9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8617,4 +8603,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>